<commit_message>
improving the model , exel sheet updation after each call
</commit_message>
<xml_diff>
--- a/data/lecture_schedule.xlsx
+++ b/data/lecture_schedule.xlsx
@@ -437,12 +437,12 @@
     <col width="10" customWidth="1" min="8" max="8"/>
     <col width="21" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
-    <col width="17" customWidth="1" min="11" max="11"/>
-    <col width="16" customWidth="1" min="12" max="12"/>
-    <col width="18" customWidth="1" min="13" max="13"/>
+    <col width="28" customWidth="1" min="11" max="11"/>
+    <col width="28" customWidth="1" min="12" max="12"/>
+    <col width="40" customWidth="1" min="13" max="13"/>
     <col width="15" customWidth="1" min="14" max="14"/>
     <col width="8" customWidth="1" min="15" max="15"/>
-    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="40" customWidth="1" min="16" max="16"/>
     <col width="23" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
@@ -536,17 +536,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>T001</t>
+          <t>T004</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Professor Amit Sharma</t>
+          <t>Dr. Sneha Reddy</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>+91-9876543210</t>
+          <t>+91-9876543213</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -556,7 +556,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Database Management Systems</t>
+          <t>Machine Learning</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -566,12 +566,12 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>10:00 AM</t>
+          <t>02:00 PM</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Lab-301</t>
+          <t>Lab-302</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -599,27 +599,27 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>T002</t>
+          <t>T005</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Dr. Priya Patel</t>
+          <t>Professor Vikram Singh</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>+91-9876543211</t>
+          <t>+91-9876543214</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Electronics</t>
+          <t>Civil</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Digital Signal Processing</t>
+          <t>Structural Analysis</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -629,12 +629,12 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>11:00 AM</t>
+          <t>03:00 PM</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Room-205</t>
+          <t>Room-110</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -725,17 +725,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>T004</t>
+          <t>T001</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Dr. Sneha Reddy</t>
+          <t>Professor Amit Sharma</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>+91-9876543213</t>
+          <t>+91-9876543210</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -745,7 +745,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Machine Learning</t>
+          <t>Database Management Systems</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -755,60 +755,82 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>02:00 PM</t>
+          <t>10:00 AM</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Lab-302</t>
+          <t>Lab-301</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Unavailable</t>
         </is>
       </c>
       <c r="J5" t="n">
         <v>0</v>
       </c>
       <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>2026-08-02T01:20:05.302240</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Assistant: Thank you for letting us know, Professor Sharma. We will record your unavailability due to being busy. Have a good day.</t>
+        </is>
+      </c>
       <c r="N5" t="n">
         <v>0</v>
       </c>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Busy</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>Assistant: Hello Professor Amit Sharma, this is the College Lecture Confirmation Assistant. I'm calling to confirm your Database Management Systems lecture scheduled for tomorrow, August 2nd, 2026, at 10:00 AM in Lab-301. Will you be available?
+Teacher: no I am not available
+Assistant: I understand. Could you please tell me the reason for your unavailability?
+Teacher: I am quiet places that I can take a lecture
+Assistant: Thank you. You mentioned you are unavailable. Could you please clarify the reason for your unavailability for tomorrow's lecture?
+Teacher: I am busy so that I am not able to take lecture
+Assistant: Thank you for letting us know, Professor Sharma. We will record your unavailability due to being busy. Have a good day.</t>
+        </is>
+      </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>T005</t>
+          <t>T002</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Professor Vikram Singh</t>
+          <t>Dr. Priya Patel</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>+91-9876543214</t>
+          <t>+91-9876543211</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Civil</t>
+          <t>Electronics</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Structural Analysis</t>
+          <t>Digital Signal Processing</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -818,33 +840,58 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>03:00 PM</t>
+          <t>11:00 AM</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Room-110</t>
+          <t>Room-205</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Unavailable</t>
         </is>
       </c>
       <c r="J6" t="n">
-        <v>0</v>
-      </c>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>2026-08-02T01:45:46.007994</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>2026-08-02T01:41:09.840116</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Assistant: Thank you for letting us know, Dr. Patel. We will make the necessary arrangements. Have a good day.</t>
+        </is>
+      </c>
       <c r="N6" t="n">
         <v>0</v>
       </c>
-      <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr"/>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>fever</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>Assistant: Hello Dr. Patel. This is the College Lecture Confirmation Assistant. I'm calling to confirm your Digital Signal Processing lecture scheduled for tomorrow, August 2nd, 2026, at 11:00 AM in Room-205. Will you be available?
+Assistant: I didn't hear you. Could you please respond?
+Teacher: no I am not available
+Assistant: I understand. Could you please tell me the reason for your unavailability?
+Teacher: I have a fever
+Assistant: Thank you for letting us know, Dr. Patel. We will make the necessary arrangements. Have a good day.</t>
+        </is>
+      </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>

</xml_diff>